<commit_message>
updates for addition to FormatCode due to new Radiology MADO code
</commit_message>
<xml_diff>
--- a/fhir/ihe.formatcode.fhir/CodeSystem-formatcode.xlsx
+++ b/fhir/ihe.formatcode.fhir/CodeSystem-formatcode.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="357">
   <si>
     <t>Property</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.4.0</t>
+    <t>1.5.1-current</t>
   </si>
   <si>
     <t>Name</t>
@@ -611,6 +611,15 @@
   </si>
   <si>
     <t>Radiology XDS-I Structured CDA</t>
+  </si>
+  <si>
+    <t>urn:ihe:rad:MADO:fhir-manifest:2026</t>
+  </si>
+  <si>
+    <t>RAD MADO</t>
+  </si>
+  <si>
+    <t>MADO Imaging Study Manifest in FHIR Format</t>
   </si>
   <si>
     <t>urn:ihe:card</t>
@@ -1469,7 +1478,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D106"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2172,7 +2181,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B53" t="s" s="2">
         <v>199</v>
@@ -2186,7 +2195,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B54" t="s" s="2">
         <v>202</v>
@@ -2242,7 +2251,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B58" t="s" s="2">
         <v>214</v>
@@ -2256,7 +2265,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B59" t="s" s="2">
         <v>217</v>
@@ -2298,7 +2307,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B62" t="s" s="2">
         <v>226</v>
@@ -2312,7 +2321,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B63" t="s" s="2">
         <v>229</v>
@@ -2326,7 +2335,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B64" t="s" s="2">
         <v>232</v>
@@ -2340,7 +2349,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B65" t="s" s="2">
         <v>235</v>
@@ -2424,7 +2433,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B71" t="s" s="2">
         <v>253</v>
@@ -2438,7 +2447,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B72" t="s" s="2">
         <v>256</v>
@@ -2788,7 +2797,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B97" t="s" s="2">
         <v>331</v>
@@ -2802,7 +2811,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B98" t="s" s="2">
         <v>334</v>
@@ -2825,7 +2834,7 @@
         <v>338</v>
       </c>
       <c r="D99" t="s" s="2">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="100">
@@ -2833,13 +2842,13 @@
         <v>63</v>
       </c>
       <c r="B100" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="C100" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="D100" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="C100" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="D100" t="s" s="2">
-        <v>336</v>
       </c>
     </row>
     <row r="101">
@@ -2847,32 +2856,32 @@
         <v>63</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C101" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D101" t="s" s="2">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C102" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D102" t="s" s="2">
-        <v>345</v>
+        <v>339</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B103" t="s" s="2">
         <v>346</v>
@@ -2892,10 +2901,10 @@
         <v>349</v>
       </c>
       <c r="C104" t="s" s="2">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D104" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="105">
@@ -2903,13 +2912,27 @@
         <v>63</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C105" t="s" s="2">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D105" t="s" s="2">
         <v>353</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s" s="2">
+        <v>63</v>
+      </c>
+      <c r="B106" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="C106" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="D106" t="s" s="2">
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates for FormatCode 1.5.0 release
</commit_message>
<xml_diff>
--- a/fhir/ihe.formatcode.fhir/CodeSystem-formatcode.xlsx
+++ b/fhir/ihe.formatcode.fhir/CodeSystem-formatcode.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="357">
   <si>
     <t>Property</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.4.0</t>
+    <t>1.5.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -611,6 +611,15 @@
   </si>
   <si>
     <t>Radiology XDS-I Structured CDA</t>
+  </si>
+  <si>
+    <t>urn:ihe:rad:MADO:fhir-manifest:2026</t>
+  </si>
+  <si>
+    <t>RAD MADO</t>
+  </si>
+  <si>
+    <t>MADO Imaging Study Manifest in FHIR Format</t>
   </si>
   <si>
     <t>urn:ihe:card</t>
@@ -1469,7 +1478,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D106"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2172,7 +2181,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B53" t="s" s="2">
         <v>199</v>
@@ -2186,7 +2195,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B54" t="s" s="2">
         <v>202</v>
@@ -2242,7 +2251,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B58" t="s" s="2">
         <v>214</v>
@@ -2256,7 +2265,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B59" t="s" s="2">
         <v>217</v>
@@ -2298,7 +2307,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B62" t="s" s="2">
         <v>226</v>
@@ -2312,7 +2321,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B63" t="s" s="2">
         <v>229</v>
@@ -2326,7 +2335,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B64" t="s" s="2">
         <v>232</v>
@@ -2340,7 +2349,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B65" t="s" s="2">
         <v>235</v>
@@ -2424,7 +2433,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B71" t="s" s="2">
         <v>253</v>
@@ -2438,7 +2447,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B72" t="s" s="2">
         <v>256</v>
@@ -2788,7 +2797,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B97" t="s" s="2">
         <v>331</v>
@@ -2802,7 +2811,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B98" t="s" s="2">
         <v>334</v>
@@ -2825,7 +2834,7 @@
         <v>338</v>
       </c>
       <c r="D99" t="s" s="2">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="100">
@@ -2833,13 +2842,13 @@
         <v>63</v>
       </c>
       <c r="B100" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="C100" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="D100" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="C100" t="s" s="2">
-        <v>340</v>
-      </c>
-      <c r="D100" t="s" s="2">
-        <v>336</v>
       </c>
     </row>
     <row r="101">
@@ -2847,32 +2856,32 @@
         <v>63</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C101" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D101" t="s" s="2">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C102" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D102" t="s" s="2">
-        <v>345</v>
+        <v>339</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B103" t="s" s="2">
         <v>346</v>
@@ -2892,10 +2901,10 @@
         <v>349</v>
       </c>
       <c r="C104" t="s" s="2">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D104" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="105">
@@ -2903,13 +2912,27 @@
         <v>63</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C105" t="s" s="2">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D105" t="s" s="2">
         <v>353</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s" s="2">
+        <v>63</v>
+      </c>
+      <c r="B106" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="C106" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="D106" t="s" s="2">
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates for FormatCode 1.6.0
</commit_message>
<xml_diff>
--- a/fhir/ihe.formatcode.fhir/CodeSystem-formatcode.xlsx
+++ b/fhir/ihe.formatcode.fhir/CodeSystem-formatcode.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="358">
   <si>
     <t>Property</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.5.0</t>
+    <t>1.6.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -299,6 +299,9 @@
   </si>
   <si>
     <t>Immunization Registry Content (IRC)</t>
+  </si>
+  <si>
+    <t>urn:ihe:pcc:ic:2009</t>
   </si>
   <si>
     <t>urn:ihe:pcc:tn:2007</t>
@@ -1478,7 +1481,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D106"/>
+  <dimension ref="A1:D107"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1667,7 +1670,7 @@
         <v>95</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D14" s="2"/>
     </row>
@@ -1676,10 +1679,10 @@
         <v>63</v>
       </c>
       <c r="B15" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="C15" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="C15" t="s" s="2">
-        <v>98</v>
       </c>
       <c r="D15" s="2"/>
     </row>
@@ -1688,10 +1691,10 @@
         <v>63</v>
       </c>
       <c r="B16" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="C16" t="s" s="2">
         <v>99</v>
-      </c>
-      <c r="C16" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="D16" s="2"/>
     </row>
@@ -1700,10 +1703,10 @@
         <v>63</v>
       </c>
       <c r="B17" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="C17" t="s" s="2">
         <v>101</v>
-      </c>
-      <c r="C17" t="s" s="2">
-        <v>102</v>
       </c>
       <c r="D17" s="2"/>
     </row>
@@ -1712,10 +1715,10 @@
         <v>63</v>
       </c>
       <c r="B18" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="C18" t="s" s="2">
         <v>103</v>
-      </c>
-      <c r="C18" t="s" s="2">
-        <v>104</v>
       </c>
       <c r="D18" s="2"/>
     </row>
@@ -1724,10 +1727,10 @@
         <v>63</v>
       </c>
       <c r="B19" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="C19" t="s" s="2">
         <v>105</v>
-      </c>
-      <c r="C19" t="s" s="2">
-        <v>106</v>
       </c>
       <c r="D19" s="2"/>
     </row>
@@ -1736,10 +1739,10 @@
         <v>63</v>
       </c>
       <c r="B20" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="C20" t="s" s="2">
         <v>107</v>
-      </c>
-      <c r="C20" t="s" s="2">
-        <v>108</v>
       </c>
       <c r="D20" s="2"/>
     </row>
@@ -1748,10 +1751,10 @@
         <v>63</v>
       </c>
       <c r="B21" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="C21" t="s" s="2">
         <v>109</v>
-      </c>
-      <c r="C21" t="s" s="2">
-        <v>110</v>
       </c>
       <c r="D21" s="2"/>
     </row>
@@ -1760,10 +1763,10 @@
         <v>63</v>
       </c>
       <c r="B22" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="C22" t="s" s="2">
         <v>111</v>
-      </c>
-      <c r="C22" t="s" s="2">
-        <v>112</v>
       </c>
       <c r="D22" s="2"/>
     </row>
@@ -1772,10 +1775,10 @@
         <v>63</v>
       </c>
       <c r="B23" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="C23" t="s" s="2">
         <v>113</v>
-      </c>
-      <c r="C23" t="s" s="2">
-        <v>114</v>
       </c>
       <c r="D23" s="2"/>
     </row>
@@ -1784,10 +1787,10 @@
         <v>63</v>
       </c>
       <c r="B24" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="C24" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="C24" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="D24" s="2"/>
     </row>
@@ -1796,10 +1799,10 @@
         <v>63</v>
       </c>
       <c r="B25" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="C25" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="C25" t="s" s="2">
-        <v>118</v>
       </c>
       <c r="D25" s="2"/>
     </row>
@@ -1808,10 +1811,10 @@
         <v>63</v>
       </c>
       <c r="B26" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="C26" t="s" s="2">
         <v>119</v>
-      </c>
-      <c r="C26" t="s" s="2">
-        <v>120</v>
       </c>
       <c r="D26" s="2"/>
     </row>
@@ -1820,27 +1823,25 @@
         <v>63</v>
       </c>
       <c r="B27" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="C27" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="C27" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="D27" t="s" s="2">
-        <v>123</v>
-      </c>
+      <c r="D27" s="2"/>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
         <v>63</v>
       </c>
       <c r="B28" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="C28" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="D28" t="s" s="2">
         <v>124</v>
-      </c>
-      <c r="C28" t="s" s="2">
-        <v>125</v>
-      </c>
-      <c r="D28" t="s" s="2">
-        <v>126</v>
       </c>
     </row>
     <row r="29">
@@ -1848,13 +1849,13 @@
         <v>63</v>
       </c>
       <c r="B29" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="C29" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="D29" t="s" s="2">
         <v>127</v>
-      </c>
-      <c r="C29" t="s" s="2">
-        <v>128</v>
-      </c>
-      <c r="D29" t="s" s="2">
-        <v>129</v>
       </c>
     </row>
     <row r="30">
@@ -1862,13 +1863,13 @@
         <v>63</v>
       </c>
       <c r="B30" t="s" s="2">
+        <v>128</v>
+      </c>
+      <c r="C30" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="D30" t="s" s="2">
         <v>130</v>
-      </c>
-      <c r="C30" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="D30" t="s" s="2">
-        <v>132</v>
       </c>
     </row>
     <row r="31">
@@ -1876,13 +1877,13 @@
         <v>63</v>
       </c>
       <c r="B31" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="C31" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="D31" t="s" s="2">
         <v>133</v>
-      </c>
-      <c r="C31" t="s" s="2">
-        <v>134</v>
-      </c>
-      <c r="D31" t="s" s="2">
-        <v>135</v>
       </c>
     </row>
     <row r="32">
@@ -1890,13 +1891,13 @@
         <v>63</v>
       </c>
       <c r="B32" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="C32" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="D32" t="s" s="2">
         <v>136</v>
-      </c>
-      <c r="C32" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="D32" t="s" s="2">
-        <v>138</v>
       </c>
     </row>
     <row r="33">
@@ -1904,13 +1905,13 @@
         <v>63</v>
       </c>
       <c r="B33" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="C33" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="D33" t="s" s="2">
         <v>139</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="D33" t="s" s="2">
-        <v>141</v>
       </c>
     </row>
     <row r="34">
@@ -1918,13 +1919,13 @@
         <v>63</v>
       </c>
       <c r="B34" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="C34" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="D34" t="s" s="2">
         <v>142</v>
-      </c>
-      <c r="C34" t="s" s="2">
-        <v>143</v>
-      </c>
-      <c r="D34" t="s" s="2">
-        <v>144</v>
       </c>
     </row>
     <row r="35">
@@ -1932,13 +1933,13 @@
         <v>63</v>
       </c>
       <c r="B35" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="C35" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="D35" t="s" s="2">
         <v>145</v>
-      </c>
-      <c r="C35" t="s" s="2">
-        <v>146</v>
-      </c>
-      <c r="D35" t="s" s="2">
-        <v>147</v>
       </c>
     </row>
     <row r="36">
@@ -1946,41 +1947,41 @@
         <v>63</v>
       </c>
       <c r="B36" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="C36" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="D36" t="s" s="2">
         <v>148</v>
-      </c>
-      <c r="C36" t="s" s="2">
-        <v>149</v>
-      </c>
-      <c r="D36" t="s" s="2">
-        <v>150</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B37" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="C37" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="D37" t="s" s="2">
         <v>151</v>
-      </c>
-      <c r="C37" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="D37" t="s" s="2">
-        <v>153</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B38" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="C38" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="D38" t="s" s="2">
         <v>154</v>
-      </c>
-      <c r="C38" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="D38" t="s" s="2">
-        <v>156</v>
       </c>
     </row>
     <row r="39">
@@ -1988,13 +1989,13 @@
         <v>63</v>
       </c>
       <c r="B39" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="C39" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="D39" t="s" s="2">
         <v>157</v>
-      </c>
-      <c r="C39" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="D39" t="s" s="2">
-        <v>159</v>
       </c>
     </row>
     <row r="40">
@@ -2002,13 +2003,13 @@
         <v>63</v>
       </c>
       <c r="B40" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="C40" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="D40" t="s" s="2">
         <v>160</v>
-      </c>
-      <c r="C40" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="D40" t="s" s="2">
-        <v>162</v>
       </c>
     </row>
     <row r="41">
@@ -2016,13 +2017,13 @@
         <v>63</v>
       </c>
       <c r="B41" t="s" s="2">
+        <v>161</v>
+      </c>
+      <c r="C41" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="D41" t="s" s="2">
         <v>163</v>
-      </c>
-      <c r="C41" t="s" s="2">
-        <v>164</v>
-      </c>
-      <c r="D41" t="s" s="2">
-        <v>165</v>
       </c>
     </row>
     <row r="42">
@@ -2030,13 +2031,13 @@
         <v>63</v>
       </c>
       <c r="B42" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="C42" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="D42" t="s" s="2">
         <v>166</v>
-      </c>
-      <c r="C42" t="s" s="2">
-        <v>167</v>
-      </c>
-      <c r="D42" t="s" s="2">
-        <v>168</v>
       </c>
     </row>
     <row r="43">
@@ -2044,13 +2045,13 @@
         <v>63</v>
       </c>
       <c r="B43" t="s" s="2">
+        <v>167</v>
+      </c>
+      <c r="C43" t="s" s="2">
+        <v>168</v>
+      </c>
+      <c r="D43" t="s" s="2">
         <v>169</v>
-      </c>
-      <c r="C43" t="s" s="2">
-        <v>170</v>
-      </c>
-      <c r="D43" t="s" s="2">
-        <v>171</v>
       </c>
     </row>
     <row r="44">
@@ -2058,13 +2059,13 @@
         <v>63</v>
       </c>
       <c r="B44" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="C44" t="s" s="2">
+        <v>171</v>
+      </c>
+      <c r="D44" t="s" s="2">
         <v>172</v>
-      </c>
-      <c r="C44" t="s" s="2">
-        <v>173</v>
-      </c>
-      <c r="D44" t="s" s="2">
-        <v>174</v>
       </c>
     </row>
     <row r="45">
@@ -2072,13 +2073,13 @@
         <v>63</v>
       </c>
       <c r="B45" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="C45" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="D45" t="s" s="2">
         <v>175</v>
-      </c>
-      <c r="C45" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="D45" t="s" s="2">
-        <v>177</v>
       </c>
     </row>
     <row r="46">
@@ -2086,69 +2087,69 @@
         <v>63</v>
       </c>
       <c r="B46" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="C46" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="D46" t="s" s="2">
         <v>178</v>
-      </c>
-      <c r="C46" t="s" s="2">
-        <v>179</v>
-      </c>
-      <c r="D46" t="s" s="2">
-        <v>180</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B47" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="C47" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="D47" t="s" s="2">
         <v>181</v>
-      </c>
-      <c r="C47" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="D47" t="s" s="2">
-        <v>183</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B48" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="C48" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="D48" t="s" s="2">
         <v>184</v>
-      </c>
-      <c r="C48" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="D48" t="s" s="2">
-        <v>186</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B49" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="C49" t="s" s="2">
+        <v>186</v>
+      </c>
+      <c r="D49" t="s" s="2">
         <v>187</v>
-      </c>
-      <c r="C49" t="s" s="2">
-        <v>188</v>
-      </c>
-      <c r="D49" t="s" s="2">
-        <v>189</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B50" t="s" s="2">
+        <v>188</v>
+      </c>
+      <c r="C50" t="s" s="2">
+        <v>189</v>
+      </c>
+      <c r="D50" t="s" s="2">
         <v>190</v>
-      </c>
-      <c r="C50" t="s" s="2">
-        <v>191</v>
-      </c>
-      <c r="D50" t="s" s="2">
-        <v>192</v>
       </c>
     </row>
     <row r="51">
@@ -2156,13 +2157,13 @@
         <v>63</v>
       </c>
       <c r="B51" t="s" s="2">
+        <v>191</v>
+      </c>
+      <c r="C51" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="D51" t="s" s="2">
         <v>193</v>
-      </c>
-      <c r="C51" t="s" s="2">
-        <v>194</v>
-      </c>
-      <c r="D51" t="s" s="2">
-        <v>195</v>
       </c>
     </row>
     <row r="52">
@@ -2170,13 +2171,13 @@
         <v>63</v>
       </c>
       <c r="B52" t="s" s="2">
+        <v>194</v>
+      </c>
+      <c r="C52" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="D52" t="s" s="2">
         <v>196</v>
-      </c>
-      <c r="C52" t="s" s="2">
-        <v>197</v>
-      </c>
-      <c r="D52" t="s" s="2">
-        <v>198</v>
       </c>
     </row>
     <row r="53">
@@ -2184,41 +2185,41 @@
         <v>63</v>
       </c>
       <c r="B53" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="C53" t="s" s="2">
+        <v>198</v>
+      </c>
+      <c r="D53" t="s" s="2">
         <v>199</v>
-      </c>
-      <c r="C53" t="s" s="2">
-        <v>200</v>
-      </c>
-      <c r="D53" t="s" s="2">
-        <v>201</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B54" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="C54" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="D54" t="s" s="2">
         <v>202</v>
-      </c>
-      <c r="C54" t="s" s="2">
-        <v>203</v>
-      </c>
-      <c r="D54" t="s" s="2">
-        <v>204</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B55" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="C55" t="s" s="2">
+        <v>204</v>
+      </c>
+      <c r="D55" t="s" s="2">
         <v>205</v>
-      </c>
-      <c r="C55" t="s" s="2">
-        <v>206</v>
-      </c>
-      <c r="D55" t="s" s="2">
-        <v>207</v>
       </c>
     </row>
     <row r="56">
@@ -2226,13 +2227,13 @@
         <v>63</v>
       </c>
       <c r="B56" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="C56" t="s" s="2">
+        <v>207</v>
+      </c>
+      <c r="D56" t="s" s="2">
         <v>208</v>
-      </c>
-      <c r="C56" t="s" s="2">
-        <v>209</v>
-      </c>
-      <c r="D56" t="s" s="2">
-        <v>210</v>
       </c>
     </row>
     <row r="57">
@@ -2240,13 +2241,13 @@
         <v>63</v>
       </c>
       <c r="B57" t="s" s="2">
+        <v>209</v>
+      </c>
+      <c r="C57" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="D57" t="s" s="2">
         <v>211</v>
-      </c>
-      <c r="C57" t="s" s="2">
-        <v>212</v>
-      </c>
-      <c r="D57" t="s" s="2">
-        <v>213</v>
       </c>
     </row>
     <row r="58">
@@ -2254,41 +2255,41 @@
         <v>63</v>
       </c>
       <c r="B58" t="s" s="2">
+        <v>212</v>
+      </c>
+      <c r="C58" t="s" s="2">
+        <v>213</v>
+      </c>
+      <c r="D58" t="s" s="2">
         <v>214</v>
-      </c>
-      <c r="C58" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="D58" t="s" s="2">
-        <v>216</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B59" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="C59" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="D59" t="s" s="2">
         <v>217</v>
-      </c>
-      <c r="C59" t="s" s="2">
-        <v>218</v>
-      </c>
-      <c r="D59" t="s" s="2">
-        <v>219</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B60" t="s" s="2">
+        <v>218</v>
+      </c>
+      <c r="C60" t="s" s="2">
+        <v>219</v>
+      </c>
+      <c r="D60" t="s" s="2">
         <v>220</v>
-      </c>
-      <c r="C60" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="D60" t="s" s="2">
-        <v>222</v>
       </c>
     </row>
     <row r="61">
@@ -2296,13 +2297,13 @@
         <v>63</v>
       </c>
       <c r="B61" t="s" s="2">
+        <v>221</v>
+      </c>
+      <c r="C61" t="s" s="2">
+        <v>222</v>
+      </c>
+      <c r="D61" t="s" s="2">
         <v>223</v>
-      </c>
-      <c r="C61" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="D61" t="s" s="2">
-        <v>225</v>
       </c>
     </row>
     <row r="62">
@@ -2310,69 +2311,69 @@
         <v>63</v>
       </c>
       <c r="B62" t="s" s="2">
+        <v>224</v>
+      </c>
+      <c r="C62" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="D62" t="s" s="2">
         <v>226</v>
-      </c>
-      <c r="C62" t="s" s="2">
-        <v>227</v>
-      </c>
-      <c r="D62" t="s" s="2">
-        <v>228</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B63" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="C63" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="D63" t="s" s="2">
         <v>229</v>
-      </c>
-      <c r="C63" t="s" s="2">
-        <v>230</v>
-      </c>
-      <c r="D63" t="s" s="2">
-        <v>231</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B64" t="s" s="2">
+        <v>230</v>
+      </c>
+      <c r="C64" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="D64" t="s" s="2">
         <v>232</v>
-      </c>
-      <c r="C64" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="D64" t="s" s="2">
-        <v>234</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B65" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="C65" t="s" s="2">
+        <v>234</v>
+      </c>
+      <c r="D65" t="s" s="2">
         <v>235</v>
-      </c>
-      <c r="C65" t="s" s="2">
-        <v>236</v>
-      </c>
-      <c r="D65" t="s" s="2">
-        <v>237</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B66" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="C66" t="s" s="2">
+        <v>237</v>
+      </c>
+      <c r="D66" t="s" s="2">
         <v>238</v>
-      </c>
-      <c r="C66" t="s" s="2">
-        <v>239</v>
-      </c>
-      <c r="D66" t="s" s="2">
-        <v>240</v>
       </c>
     </row>
     <row r="67">
@@ -2380,13 +2381,13 @@
         <v>63</v>
       </c>
       <c r="B67" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="C67" t="s" s="2">
+        <v>240</v>
+      </c>
+      <c r="D67" t="s" s="2">
         <v>241</v>
-      </c>
-      <c r="C67" t="s" s="2">
-        <v>242</v>
-      </c>
-      <c r="D67" t="s" s="2">
-        <v>243</v>
       </c>
     </row>
     <row r="68">
@@ -2394,13 +2395,13 @@
         <v>63</v>
       </c>
       <c r="B68" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="C68" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="D68" t="s" s="2">
         <v>244</v>
-      </c>
-      <c r="C68" t="s" s="2">
-        <v>245</v>
-      </c>
-      <c r="D68" t="s" s="2">
-        <v>246</v>
       </c>
     </row>
     <row r="69">
@@ -2408,13 +2409,13 @@
         <v>63</v>
       </c>
       <c r="B69" t="s" s="2">
+        <v>245</v>
+      </c>
+      <c r="C69" t="s" s="2">
+        <v>246</v>
+      </c>
+      <c r="D69" t="s" s="2">
         <v>247</v>
-      </c>
-      <c r="C69" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="D69" t="s" s="2">
-        <v>249</v>
       </c>
     </row>
     <row r="70">
@@ -2422,13 +2423,13 @@
         <v>63</v>
       </c>
       <c r="B70" t="s" s="2">
+        <v>248</v>
+      </c>
+      <c r="C70" t="s" s="2">
+        <v>249</v>
+      </c>
+      <c r="D70" t="s" s="2">
         <v>250</v>
-      </c>
-      <c r="C70" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="D70" t="s" s="2">
-        <v>252</v>
       </c>
     </row>
     <row r="71">
@@ -2436,41 +2437,41 @@
         <v>63</v>
       </c>
       <c r="B71" t="s" s="2">
+        <v>251</v>
+      </c>
+      <c r="C71" t="s" s="2">
+        <v>252</v>
+      </c>
+      <c r="D71" t="s" s="2">
         <v>253</v>
-      </c>
-      <c r="C71" t="s" s="2">
-        <v>254</v>
-      </c>
-      <c r="D71" t="s" s="2">
-        <v>255</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B72" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="C72" t="s" s="2">
+        <v>255</v>
+      </c>
+      <c r="D72" t="s" s="2">
         <v>256</v>
-      </c>
-      <c r="C72" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="D72" t="s" s="2">
-        <v>258</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B73" t="s" s="2">
+        <v>257</v>
+      </c>
+      <c r="C73" t="s" s="2">
+        <v>258</v>
+      </c>
+      <c r="D73" t="s" s="2">
         <v>259</v>
-      </c>
-      <c r="C73" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="D73" t="s" s="2">
-        <v>261</v>
       </c>
     </row>
     <row r="74">
@@ -2478,13 +2479,13 @@
         <v>63</v>
       </c>
       <c r="B74" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="C74" t="s" s="2">
+        <v>261</v>
+      </c>
+      <c r="D74" t="s" s="2">
         <v>262</v>
-      </c>
-      <c r="C74" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="D74" t="s" s="2">
-        <v>264</v>
       </c>
     </row>
     <row r="75">
@@ -2492,13 +2493,13 @@
         <v>63</v>
       </c>
       <c r="B75" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="C75" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="D75" t="s" s="2">
         <v>265</v>
-      </c>
-      <c r="C75" t="s" s="2">
-        <v>266</v>
-      </c>
-      <c r="D75" t="s" s="2">
-        <v>267</v>
       </c>
     </row>
     <row r="76">
@@ -2506,13 +2507,13 @@
         <v>63</v>
       </c>
       <c r="B76" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="C76" t="s" s="2">
+        <v>267</v>
+      </c>
+      <c r="D76" t="s" s="2">
         <v>268</v>
-      </c>
-      <c r="C76" t="s" s="2">
-        <v>269</v>
-      </c>
-      <c r="D76" t="s" s="2">
-        <v>270</v>
       </c>
     </row>
     <row r="77">
@@ -2520,13 +2521,13 @@
         <v>63</v>
       </c>
       <c r="B77" t="s" s="2">
+        <v>269</v>
+      </c>
+      <c r="C77" t="s" s="2">
+        <v>270</v>
+      </c>
+      <c r="D77" t="s" s="2">
         <v>271</v>
-      </c>
-      <c r="C77" t="s" s="2">
-        <v>272</v>
-      </c>
-      <c r="D77" t="s" s="2">
-        <v>273</v>
       </c>
     </row>
     <row r="78">
@@ -2534,13 +2535,13 @@
         <v>63</v>
       </c>
       <c r="B78" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="C78" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="D78" t="s" s="2">
         <v>274</v>
-      </c>
-      <c r="C78" t="s" s="2">
-        <v>275</v>
-      </c>
-      <c r="D78" t="s" s="2">
-        <v>276</v>
       </c>
     </row>
     <row r="79">
@@ -2548,13 +2549,13 @@
         <v>63</v>
       </c>
       <c r="B79" t="s" s="2">
+        <v>275</v>
+      </c>
+      <c r="C79" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="D79" t="s" s="2">
         <v>277</v>
-      </c>
-      <c r="C79" t="s" s="2">
-        <v>278</v>
-      </c>
-      <c r="D79" t="s" s="2">
-        <v>279</v>
       </c>
     </row>
     <row r="80">
@@ -2562,13 +2563,13 @@
         <v>63</v>
       </c>
       <c r="B80" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="C80" t="s" s="2">
+        <v>279</v>
+      </c>
+      <c r="D80" t="s" s="2">
         <v>280</v>
-      </c>
-      <c r="C80" t="s" s="2">
-        <v>281</v>
-      </c>
-      <c r="D80" t="s" s="2">
-        <v>282</v>
       </c>
     </row>
     <row r="81">
@@ -2576,13 +2577,13 @@
         <v>63</v>
       </c>
       <c r="B81" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="C81" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="D81" t="s" s="2">
         <v>283</v>
-      </c>
-      <c r="C81" t="s" s="2">
-        <v>284</v>
-      </c>
-      <c r="D81" t="s" s="2">
-        <v>285</v>
       </c>
     </row>
     <row r="82">
@@ -2590,13 +2591,13 @@
         <v>63</v>
       </c>
       <c r="B82" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="C82" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="D82" t="s" s="2">
         <v>286</v>
-      </c>
-      <c r="C82" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="D82" t="s" s="2">
-        <v>288</v>
       </c>
     </row>
     <row r="83">
@@ -2604,13 +2605,13 @@
         <v>63</v>
       </c>
       <c r="B83" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="C83" t="s" s="2">
+        <v>288</v>
+      </c>
+      <c r="D83" t="s" s="2">
         <v>289</v>
-      </c>
-      <c r="C83" t="s" s="2">
-        <v>290</v>
-      </c>
-      <c r="D83" t="s" s="2">
-        <v>291</v>
       </c>
     </row>
     <row r="84">
@@ -2618,13 +2619,13 @@
         <v>63</v>
       </c>
       <c r="B84" t="s" s="2">
+        <v>290</v>
+      </c>
+      <c r="C84" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="D84" t="s" s="2">
         <v>292</v>
-      </c>
-      <c r="C84" t="s" s="2">
-        <v>293</v>
-      </c>
-      <c r="D84" t="s" s="2">
-        <v>294</v>
       </c>
     </row>
     <row r="85">
@@ -2632,13 +2633,13 @@
         <v>63</v>
       </c>
       <c r="B85" t="s" s="2">
+        <v>293</v>
+      </c>
+      <c r="C85" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="D85" t="s" s="2">
         <v>295</v>
-      </c>
-      <c r="C85" t="s" s="2">
-        <v>296</v>
-      </c>
-      <c r="D85" t="s" s="2">
-        <v>297</v>
       </c>
     </row>
     <row r="86">
@@ -2646,13 +2647,13 @@
         <v>63</v>
       </c>
       <c r="B86" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="C86" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="D86" t="s" s="2">
         <v>298</v>
-      </c>
-      <c r="C86" t="s" s="2">
-        <v>299</v>
-      </c>
-      <c r="D86" t="s" s="2">
-        <v>300</v>
       </c>
     </row>
     <row r="87">
@@ -2660,13 +2661,13 @@
         <v>63</v>
       </c>
       <c r="B87" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="C87" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="D87" t="s" s="2">
         <v>301</v>
-      </c>
-      <c r="C87" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="D87" t="s" s="2">
-        <v>303</v>
       </c>
     </row>
     <row r="88">
@@ -2674,13 +2675,13 @@
         <v>63</v>
       </c>
       <c r="B88" t="s" s="2">
+        <v>302</v>
+      </c>
+      <c r="C88" t="s" s="2">
+        <v>303</v>
+      </c>
+      <c r="D88" t="s" s="2">
         <v>304</v>
-      </c>
-      <c r="C88" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="D88" t="s" s="2">
-        <v>306</v>
       </c>
     </row>
     <row r="89">
@@ -2688,13 +2689,13 @@
         <v>63</v>
       </c>
       <c r="B89" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="C89" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="D89" t="s" s="2">
         <v>307</v>
-      </c>
-      <c r="C89" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="D89" t="s" s="2">
-        <v>309</v>
       </c>
     </row>
     <row r="90">
@@ -2702,13 +2703,13 @@
         <v>63</v>
       </c>
       <c r="B90" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="C90" t="s" s="2">
+        <v>309</v>
+      </c>
+      <c r="D90" t="s" s="2">
         <v>310</v>
-      </c>
-      <c r="C90" t="s" s="2">
-        <v>311</v>
-      </c>
-      <c r="D90" t="s" s="2">
-        <v>312</v>
       </c>
     </row>
     <row r="91">
@@ -2716,13 +2717,13 @@
         <v>63</v>
       </c>
       <c r="B91" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="C91" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="D91" t="s" s="2">
         <v>313</v>
-      </c>
-      <c r="C91" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="D91" t="s" s="2">
-        <v>315</v>
       </c>
     </row>
     <row r="92">
@@ -2730,13 +2731,13 @@
         <v>63</v>
       </c>
       <c r="B92" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="C92" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="D92" t="s" s="2">
         <v>316</v>
-      </c>
-      <c r="C92" t="s" s="2">
-        <v>317</v>
-      </c>
-      <c r="D92" t="s" s="2">
-        <v>318</v>
       </c>
     </row>
     <row r="93">
@@ -2744,13 +2745,13 @@
         <v>63</v>
       </c>
       <c r="B93" t="s" s="2">
+        <v>317</v>
+      </c>
+      <c r="C93" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="D93" t="s" s="2">
         <v>319</v>
-      </c>
-      <c r="C93" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="D93" t="s" s="2">
-        <v>321</v>
       </c>
     </row>
     <row r="94">
@@ -2758,13 +2759,13 @@
         <v>63</v>
       </c>
       <c r="B94" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="C94" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="D94" t="s" s="2">
         <v>322</v>
-      </c>
-      <c r="C94" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="D94" t="s" s="2">
-        <v>324</v>
       </c>
     </row>
     <row r="95">
@@ -2772,13 +2773,13 @@
         <v>63</v>
       </c>
       <c r="B95" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="C95" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="D95" t="s" s="2">
         <v>325</v>
-      </c>
-      <c r="C95" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="D95" t="s" s="2">
-        <v>327</v>
       </c>
     </row>
     <row r="96">
@@ -2786,13 +2787,13 @@
         <v>63</v>
       </c>
       <c r="B96" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="C96" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="D96" t="s" s="2">
         <v>328</v>
-      </c>
-      <c r="C96" t="s" s="2">
-        <v>329</v>
-      </c>
-      <c r="D96" t="s" s="2">
-        <v>330</v>
       </c>
     </row>
     <row r="97">
@@ -2800,41 +2801,41 @@
         <v>63</v>
       </c>
       <c r="B97" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="C97" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="D97" t="s" s="2">
         <v>331</v>
-      </c>
-      <c r="C97" t="s" s="2">
-        <v>332</v>
-      </c>
-      <c r="D97" t="s" s="2">
-        <v>333</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B98" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="C98" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="D98" t="s" s="2">
         <v>334</v>
-      </c>
-      <c r="C98" t="s" s="2">
-        <v>335</v>
-      </c>
-      <c r="D98" t="s" s="2">
-        <v>336</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B99" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="C99" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="D99" t="s" s="2">
         <v>337</v>
-      </c>
-      <c r="C99" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="D99" t="s" s="2">
-        <v>339</v>
       </c>
     </row>
     <row r="100">
@@ -2842,13 +2843,13 @@
         <v>63</v>
       </c>
       <c r="B100" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="C100" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="D100" t="s" s="2">
         <v>340</v>
-      </c>
-      <c r="C100" t="s" s="2">
-        <v>341</v>
-      </c>
-      <c r="D100" t="s" s="2">
-        <v>339</v>
       </c>
     </row>
     <row r="101">
@@ -2856,13 +2857,13 @@
         <v>63</v>
       </c>
       <c r="B101" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="C101" t="s" s="2">
         <v>342</v>
       </c>
-      <c r="C101" t="s" s="2">
-        <v>343</v>
-      </c>
       <c r="D101" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="102">
@@ -2870,41 +2871,41 @@
         <v>63</v>
       </c>
       <c r="B102" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="C102" t="s" s="2">
         <v>344</v>
       </c>
-      <c r="C102" t="s" s="2">
-        <v>345</v>
-      </c>
       <c r="D102" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B103" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="C103" t="s" s="2">
         <v>346</v>
       </c>
-      <c r="C103" t="s" s="2">
-        <v>347</v>
-      </c>
       <c r="D103" t="s" s="2">
-        <v>348</v>
+        <v>340</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B104" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="C104" t="s" s="2">
+        <v>348</v>
+      </c>
+      <c r="D104" t="s" s="2">
         <v>349</v>
-      </c>
-      <c r="C104" t="s" s="2">
-        <v>350</v>
-      </c>
-      <c r="D104" t="s" s="2">
-        <v>351</v>
       </c>
     </row>
     <row r="105">
@@ -2912,13 +2913,13 @@
         <v>63</v>
       </c>
       <c r="B105" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="C105" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="D105" t="s" s="2">
         <v>352</v>
-      </c>
-      <c r="C105" t="s" s="2">
-        <v>350</v>
-      </c>
-      <c r="D105" t="s" s="2">
-        <v>353</v>
       </c>
     </row>
     <row r="106">
@@ -2926,13 +2927,27 @@
         <v>63</v>
       </c>
       <c r="B106" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="C106" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="D106" t="s" s="2">
         <v>354</v>
       </c>
-      <c r="C106" t="s" s="2">
+    </row>
+    <row r="107">
+      <c r="A107" t="s" s="2">
+        <v>63</v>
+      </c>
+      <c r="B107" t="s" s="2">
         <v>355</v>
       </c>
-      <c r="D106" t="s" s="2">
+      <c r="C107" t="s" s="2">
         <v>356</v>
+      </c>
+      <c r="D107" t="s" s="2">
+        <v>357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>